<commit_message>
Record 03.08.2026 T1 attendance in the workbook
Transcribed from the marked printout: 28 of 31 students present.
Salvi Aniket Bharat, Murala Vamshi and Ashish Sinha have no mark on the
physical sheet, so their cells are left blank rather than inferred as
absent (per TA's call), and are excluded from the TOTAL PRESENT count.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8xm6SyckYLxZx63RYxYRb
</commit_message>
<xml_diff>
--- a/attendance/BB101_T1_Attendance.xlsx
+++ b/attendance/BB101_T1_Attendance.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,11 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -70,7 +75,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -204,11 +209,121 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -263,6 +378,13 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -687,10 +809,14 @@
       <c r="J3" s="7" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="10" t="n"/>
+      <c r="A4" s="25" t="n"/>
+      <c r="B4" s="26" t="n"/>
+      <c r="C4" s="26" t="n"/>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>03.08.2026</t>
+        </is>
+      </c>
       <c r="E4" s="11" t="n"/>
       <c r="F4" s="11" t="n"/>
       <c r="G4" s="11" t="n"/>
@@ -756,7 +882,11 @@
           <t>Kadem Akhil</t>
         </is>
       </c>
-      <c r="D7" s="16" t="n"/>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E7" s="17" t="n"/>
       <c r="F7" s="17" t="n"/>
       <c r="G7" s="17" t="n"/>
@@ -778,7 +908,11 @@
           <t>Vedant Nitin Deshmukh</t>
         </is>
       </c>
-      <c r="D8" s="16" t="n"/>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E8" s="17" t="n"/>
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="17" t="n"/>
@@ -800,7 +934,11 @@
           <t>Chetaansi Mina</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n"/>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="n"/>
       <c r="F9" s="17" t="n"/>
       <c r="G9" s="17" t="n"/>
@@ -822,7 +960,11 @@
           <t>Aashna Shetty</t>
         </is>
       </c>
-      <c r="D10" s="16" t="n"/>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E10" s="17" t="n"/>
       <c r="F10" s="17" t="n"/>
       <c r="G10" s="17" t="n"/>
@@ -844,7 +986,11 @@
           <t>Ananya Krishna Jakka</t>
         </is>
       </c>
-      <c r="D11" s="16" t="n"/>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E11" s="17" t="n"/>
       <c r="F11" s="17" t="n"/>
       <c r="G11" s="17" t="n"/>
@@ -888,7 +1034,11 @@
           <t>Bhargav Dhananjay Gawale</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n"/>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E13" s="17" t="n"/>
       <c r="F13" s="17" t="n"/>
       <c r="G13" s="17" t="n"/>
@@ -910,7 +1060,11 @@
           <t>Dhruv Hemant Savla</t>
         </is>
       </c>
-      <c r="D14" s="16" t="n"/>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E14" s="17" t="n"/>
       <c r="F14" s="17" t="n"/>
       <c r="G14" s="17" t="n"/>
@@ -932,7 +1086,11 @@
           <t>Gayatri Bishnoi</t>
         </is>
       </c>
-      <c r="D15" s="16" t="n"/>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E15" s="17" t="n"/>
       <c r="F15" s="17" t="n"/>
       <c r="G15" s="17" t="n"/>
@@ -954,7 +1112,11 @@
           <t>Ishank Reddy Tatipalli</t>
         </is>
       </c>
-      <c r="D16" s="16" t="n"/>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E16" s="17" t="n"/>
       <c r="F16" s="17" t="n"/>
       <c r="G16" s="17" t="n"/>
@@ -976,7 +1138,11 @@
           <t>Jitesh Sanjay Thakur</t>
         </is>
       </c>
-      <c r="D17" s="16" t="n"/>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E17" s="17" t="n"/>
       <c r="F17" s="17" t="n"/>
       <c r="G17" s="17" t="n"/>
@@ -998,7 +1164,11 @@
           <t>Laksh Vinod Rampurkar</t>
         </is>
       </c>
-      <c r="D18" s="16" t="n"/>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E18" s="17" t="n"/>
       <c r="F18" s="17" t="n"/>
       <c r="G18" s="17" t="n"/>
@@ -1020,7 +1190,11 @@
           <t>Mayank Meena</t>
         </is>
       </c>
-      <c r="D19" s="16" t="n"/>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E19" s="17" t="n"/>
       <c r="F19" s="17" t="n"/>
       <c r="G19" s="17" t="n"/>
@@ -1042,7 +1216,11 @@
           <t>Mishti Khandelwal</t>
         </is>
       </c>
-      <c r="D20" s="16" t="n"/>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E20" s="17" t="n"/>
       <c r="F20" s="17" t="n"/>
       <c r="G20" s="17" t="n"/>
@@ -1064,7 +1242,11 @@
           <t>Nishit Katole</t>
         </is>
       </c>
-      <c r="D21" s="16" t="n"/>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E21" s="17" t="n"/>
       <c r="F21" s="17" t="n"/>
       <c r="G21" s="17" t="n"/>
@@ -1086,7 +1268,11 @@
           <t>Patel Vishw Dilipkumar</t>
         </is>
       </c>
-      <c r="D22" s="16" t="n"/>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E22" s="17" t="n"/>
       <c r="F22" s="17" t="n"/>
       <c r="G22" s="17" t="n"/>
@@ -1108,7 +1294,11 @@
           <t>Prasad Manjukumari Brijesh</t>
         </is>
       </c>
-      <c r="D23" s="16" t="n"/>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E23" s="17" t="n"/>
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="17" t="n"/>
@@ -1130,7 +1320,11 @@
           <t>Rishabh Gupta</t>
         </is>
       </c>
-      <c r="D24" s="16" t="n"/>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E24" s="17" t="n"/>
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="17" t="n"/>
@@ -1152,7 +1346,11 @@
           <t>Sajil Suryawanshi</t>
         </is>
       </c>
-      <c r="D25" s="16" t="n"/>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E25" s="17" t="n"/>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="17" t="n"/>
@@ -1174,7 +1372,11 @@
           <t>Sarje Yashraaj Balaji</t>
         </is>
       </c>
-      <c r="D26" s="16" t="n"/>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E26" s="17" t="n"/>
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="17" t="n"/>
@@ -1196,7 +1398,11 @@
           <t>Shashank Gupta</t>
         </is>
       </c>
-      <c r="D27" s="16" t="n"/>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E27" s="17" t="n"/>
       <c r="F27" s="17" t="n"/>
       <c r="G27" s="17" t="n"/>
@@ -1218,7 +1424,11 @@
           <t>Sukrit Majumdar</t>
         </is>
       </c>
-      <c r="D28" s="16" t="n"/>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E28" s="17" t="n"/>
       <c r="F28" s="17" t="n"/>
       <c r="G28" s="17" t="n"/>
@@ -1240,7 +1450,11 @@
           <t>Tegjyot Singh</t>
         </is>
       </c>
-      <c r="D29" s="16" t="n"/>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E29" s="17" t="n"/>
       <c r="F29" s="17" t="n"/>
       <c r="G29" s="17" t="n"/>
@@ -1262,7 +1476,11 @@
           <t>Vihaan Kamdar</t>
         </is>
       </c>
-      <c r="D30" s="16" t="n"/>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
       <c r="G30" s="17" t="n"/>
@@ -1284,7 +1502,11 @@
           <t>Yashita Prakash</t>
         </is>
       </c>
-      <c r="D31" s="16" t="n"/>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E31" s="17" t="n"/>
       <c r="F31" s="17" t="n"/>
       <c r="G31" s="17" t="n"/>
@@ -1306,7 +1528,11 @@
           <t>Aditika Kamal</t>
         </is>
       </c>
-      <c r="D32" s="16" t="n"/>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E32" s="17" t="n"/>
       <c r="F32" s="17" t="n"/>
       <c r="G32" s="17" t="n"/>
@@ -1328,7 +1554,11 @@
           <t>Gourinandan A Pai</t>
         </is>
       </c>
-      <c r="D33" s="16" t="n"/>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E33" s="17" t="n"/>
       <c r="F33" s="17" t="n"/>
       <c r="G33" s="17" t="n"/>
@@ -1350,7 +1580,11 @@
           <t>Priyanshu Raj</t>
         </is>
       </c>
-      <c r="D34" s="16" t="n"/>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E34" s="17" t="n"/>
       <c r="F34" s="17" t="n"/>
       <c r="G34" s="17" t="n"/>
@@ -1372,7 +1606,11 @@
           <t>Sunkara Akhila Sai</t>
         </is>
       </c>
-      <c r="D35" s="16" t="n"/>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="E35" s="17" t="n"/>
       <c r="F35" s="17" t="n"/>
       <c r="G35" s="17" t="n"/>
@@ -1386,8 +1624,8 @@
           <t>TOTAL PRESENT</t>
         </is>
       </c>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="20" t="n"/>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="28" t="n"/>
       <c r="D36" s="21">
         <f>IF(COUNTA(D5:D35)=0,"",COUNTIF(D5:D35,"P"))</f>
         <v/>

</xml_diff>

<commit_message>
Record 10.08.2026 attendance and add group assignments
Fills the second date column in both the standalone attendance sheet
and the combined tracker. Adds a Groups tab (Group 1 self-formed from
the students, Groups 2-3 split at random from the rest of the roster)
and wires the group name into the Extempore Grading sheet's Group
column automatically.
</commit_message>
<xml_diff>
--- a/attendance/BB101_T1_Attendance.xlsx
+++ b/attendance/BB101_T1_Attendance.xlsx
@@ -323,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -384,6 +384,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -817,7 +820,11 @@
           <t>03.08.2026</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n"/>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>10.08.2026</t>
+        </is>
+      </c>
       <c r="F4" s="11" t="n"/>
       <c r="G4" s="11" t="n"/>
       <c r="H4" s="11" t="n"/>
@@ -913,7 +920,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E8" s="17" t="n"/>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="17" t="n"/>
       <c r="H8" s="17" t="n"/>
@@ -939,7 +950,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E9" s="17" t="n"/>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F9" s="17" t="n"/>
       <c r="G9" s="17" t="n"/>
       <c r="H9" s="17" t="n"/>
@@ -965,7 +980,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E10" s="17" t="n"/>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F10" s="17" t="n"/>
       <c r="G10" s="17" t="n"/>
       <c r="H10" s="17" t="n"/>
@@ -991,7 +1010,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E11" s="17" t="n"/>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F11" s="17" t="n"/>
       <c r="G11" s="17" t="n"/>
       <c r="H11" s="17" t="n"/>
@@ -1013,7 +1036,11 @@
         </is>
       </c>
       <c r="D12" s="16" t="n"/>
-      <c r="E12" s="17" t="n"/>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F12" s="17" t="n"/>
       <c r="G12" s="17" t="n"/>
       <c r="H12" s="17" t="n"/>
@@ -1039,7 +1066,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E13" s="17" t="n"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F13" s="17" t="n"/>
       <c r="G13" s="17" t="n"/>
       <c r="H13" s="17" t="n"/>
@@ -1065,7 +1096,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E14" s="17" t="n"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F14" s="17" t="n"/>
       <c r="G14" s="17" t="n"/>
       <c r="H14" s="17" t="n"/>
@@ -1091,7 +1126,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n"/>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F15" s="17" t="n"/>
       <c r="G15" s="17" t="n"/>
       <c r="H15" s="17" t="n"/>
@@ -1117,7 +1156,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E16" s="17" t="n"/>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F16" s="17" t="n"/>
       <c r="G16" s="17" t="n"/>
       <c r="H16" s="17" t="n"/>
@@ -1143,7 +1186,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E17" s="17" t="n"/>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F17" s="17" t="n"/>
       <c r="G17" s="17" t="n"/>
       <c r="H17" s="17" t="n"/>
@@ -1169,7 +1216,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E18" s="17" t="n"/>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F18" s="17" t="n"/>
       <c r="G18" s="17" t="n"/>
       <c r="H18" s="17" t="n"/>
@@ -1195,7 +1246,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E19" s="17" t="n"/>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F19" s="17" t="n"/>
       <c r="G19" s="17" t="n"/>
       <c r="H19" s="17" t="n"/>
@@ -1221,7 +1276,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E20" s="17" t="n"/>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F20" s="17" t="n"/>
       <c r="G20" s="17" t="n"/>
       <c r="H20" s="17" t="n"/>
@@ -1247,7 +1306,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E21" s="17" t="n"/>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F21" s="17" t="n"/>
       <c r="G21" s="17" t="n"/>
       <c r="H21" s="17" t="n"/>
@@ -1273,7 +1336,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n"/>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F22" s="17" t="n"/>
       <c r="G22" s="17" t="n"/>
       <c r="H22" s="17" t="n"/>
@@ -1299,7 +1366,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n"/>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="17" t="n"/>
       <c r="H23" s="17" t="n"/>
@@ -1325,7 +1396,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E24" s="17" t="n"/>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="17" t="n"/>
       <c r="H24" s="17" t="n"/>
@@ -1351,7 +1426,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E25" s="17" t="n"/>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="17" t="n"/>
       <c r="H25" s="17" t="n"/>
@@ -1377,7 +1456,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E26" s="17" t="n"/>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="17" t="n"/>
       <c r="H26" s="17" t="n"/>
@@ -1403,7 +1486,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E27" s="17" t="n"/>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F27" s="17" t="n"/>
       <c r="G27" s="17" t="n"/>
       <c r="H27" s="17" t="n"/>
@@ -1429,7 +1516,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E28" s="17" t="n"/>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F28" s="17" t="n"/>
       <c r="G28" s="17" t="n"/>
       <c r="H28" s="17" t="n"/>
@@ -1455,7 +1546,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E29" s="17" t="n"/>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F29" s="17" t="n"/>
       <c r="G29" s="17" t="n"/>
       <c r="H29" s="17" t="n"/>
@@ -1481,7 +1576,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E30" s="17" t="n"/>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F30" s="17" t="n"/>
       <c r="G30" s="17" t="n"/>
       <c r="H30" s="17" t="n"/>
@@ -1507,7 +1606,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E31" s="17" t="n"/>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F31" s="17" t="n"/>
       <c r="G31" s="17" t="n"/>
       <c r="H31" s="17" t="n"/>
@@ -1533,7 +1636,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E32" s="17" t="n"/>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F32" s="17" t="n"/>
       <c r="G32" s="17" t="n"/>
       <c r="H32" s="17" t="n"/>
@@ -1559,7 +1666,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E33" s="17" t="n"/>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F33" s="17" t="n"/>
       <c r="G33" s="17" t="n"/>
       <c r="H33" s="17" t="n"/>
@@ -1585,7 +1696,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E34" s="17" t="n"/>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F34" s="17" t="n"/>
       <c r="G34" s="17" t="n"/>
       <c r="H34" s="17" t="n"/>
@@ -1611,7 +1726,11 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E35" s="17" t="n"/>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="F35" s="17" t="n"/>
       <c r="G35" s="17" t="n"/>
       <c r="H35" s="17" t="n"/>

</xml_diff>